<commit_message>
chore(drive): sync Drive data files and add Cronograma xlsx
Re-synced existing Drive files via rclone and added new assets:
- Cronograma actual.xlsx (updated schedule with real dates)
- evaluacion_economica_bebidas_carbonatadas_v2.pdf
- Archivos página/ folder with project assets
- Diagramas de operaciones/ folder
- CocaCola400mL 1.0.spp (Tecnomatix simulation)
- APM.ods project tracker
</commit_message>
<xml_diff>
--- a/archivos-drive/DAP.xlsx
+++ b/archivos-drive/DAP.xlsx
@@ -31,7 +31,7 @@
     <t>Operación</t>
   </si>
   <si>
-    <t>Operación: Embotellado de Coca-Cola 400ml retornable</t>
+    <t>Operación: Embotellado de Gaseosa 400ml retornable</t>
   </si>
   <si>
     <t>➪</t>
@@ -1014,7 +1014,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1034,8 +1034,8 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -1091,6 +1091,9 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -2424,7 +2427,7 @@
       <c r="B35" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="29" t="s">
         <v>77</v>
       </c>
       <c r="D35" s="3"/>
@@ -2442,7 +2445,7 @@
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="B36" s="29"/>
+      <c r="B36" s="30"/>
       <c r="C36" s="11" t="s">
         <v>8</v>
       </c>
@@ -2601,21 +2604,21 @@
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="30"/>
+      <c r="A42" s="31"/>
       <c r="B42" s="16">
         <v>5.0</v>
       </c>
-      <c r="C42" s="31" t="s">
+      <c r="C42" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="D42" s="31" t="s">
+      <c r="D42" s="32" t="s">
         <v>37</v>
       </c>
       <c r="E42" s="1"/>
-      <c r="F42" s="32">
+      <c r="F42" s="33">
         <v>60.0</v>
       </c>
-      <c r="G42" s="33" t="s">
+      <c r="G42" s="34" t="s">
         <v>24</v>
       </c>
       <c r="H42" s="1"/>
@@ -2623,20 +2626,20 @@
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
-      <c r="M42" s="30"/>
-      <c r="N42" s="30"/>
-      <c r="O42" s="30"/>
-      <c r="P42" s="30"/>
-      <c r="Q42" s="30"/>
-      <c r="R42" s="30"/>
-      <c r="S42" s="30"/>
-      <c r="T42" s="30"/>
-      <c r="U42" s="30"/>
-      <c r="V42" s="30"/>
-      <c r="W42" s="30"/>
-      <c r="X42" s="30"/>
-      <c r="Y42" s="30"/>
-      <c r="Z42" s="30"/>
+      <c r="M42" s="31"/>
+      <c r="N42" s="31"/>
+      <c r="O42" s="31"/>
+      <c r="P42" s="31"/>
+      <c r="Q42" s="31"/>
+      <c r="R42" s="31"/>
+      <c r="S42" s="31"/>
+      <c r="T42" s="31"/>
+      <c r="U42" s="31"/>
+      <c r="V42" s="31"/>
+      <c r="W42" s="31"/>
+      <c r="X42" s="31"/>
+      <c r="Y42" s="31"/>
+      <c r="Z42" s="31"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="B43" s="16">
@@ -2691,7 +2694,7 @@
       <c r="B45" s="16">
         <v>8.0</v>
       </c>
-      <c r="C45" s="34" t="s">
+      <c r="C45" s="35" t="s">
         <v>84</v>
       </c>
       <c r="D45" s="17" t="s">
@@ -3124,7 +3127,7 @@
       <c r="B64" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="29" t="s">
         <v>107</v>
       </c>
       <c r="D64" s="3"/>
@@ -3141,7 +3144,7 @@
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="B65" s="29"/>
+      <c r="B65" s="30"/>
       <c r="C65" s="11" t="s">
         <v>8</v>
       </c>
@@ -3356,7 +3359,7 @@
       <c r="B73" s="16">
         <v>7.0</v>
       </c>
-      <c r="C73" s="34" t="s">
+      <c r="C73" s="35" t="s">
         <v>117</v>
       </c>
       <c r="D73" s="17" t="s">
@@ -4598,6 +4601,9 @@
     <row r="1008" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="N13:S13"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:L2"/>
     <mergeCell ref="C3:E3"/>
@@ -4605,27 +4611,24 @@
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="D65:D66"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="L36:L37"/>
-    <mergeCell ref="F63:L63"/>
-    <mergeCell ref="F64:L64"/>
-    <mergeCell ref="G65:K65"/>
-    <mergeCell ref="L65:L66"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="L4:L5"/>
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="F34:L34"/>
     <mergeCell ref="B35:B37"/>
     <mergeCell ref="C35:E35"/>
     <mergeCell ref="F35:L35"/>
-    <mergeCell ref="N13:S13"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="D65:D66"/>
+    <mergeCell ref="G65:K65"/>
+    <mergeCell ref="L65:L66"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="L36:L37"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="F63:L63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="F64:L64"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.25" right="0.25" top="0.75"/>
@@ -4682,7 +4685,7 @@
       <c r="C4" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="35">
+      <c r="D4" s="36">
         <v>3600.0</v>
       </c>
       <c r="E4" s="27" t="s">
@@ -4702,7 +4705,7 @@
       <c r="C5" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="35">
+      <c r="D5" s="36">
         <v>20000.0</v>
       </c>
       <c r="E5" s="27" t="s">
@@ -4722,7 +4725,7 @@
       <c r="C6" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="36">
+      <c r="D6" s="37">
         <f>D4/D5</f>
         <v>0.18</v>
       </c>
@@ -4737,27 +4740,27 @@
       </c>
     </row>
     <row r="7" ht="157.5" customHeight="1">
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="38" t="s">
         <v>148</v>
       </c>
-      <c r="D7" s="35">
+      <c r="D7" s="36">
         <v>0.1</v>
       </c>
-      <c r="E7" s="37" t="s">
+      <c r="E7" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="F7" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="37">
+      <c r="G7" s="40"/>
+      <c r="H7" s="38">
         <f>(391-255)/1440</f>
         <v>0.09444444444</v>
       </c>
-      <c r="I7" s="40" t="s">
+      <c r="I7" s="41" t="s">
         <v>150</v>
       </c>
     </row>
@@ -4768,13 +4771,13 @@
       <c r="C8" s="27" t="s">
         <v>152</v>
       </c>
-      <c r="D8" s="35">
+      <c r="D8" s="36">
         <v>0.03</v>
       </c>
       <c r="E8" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="41" t="s">
         <v>153</v>
       </c>
     </row>
@@ -4785,13 +4788,13 @@
       <c r="C9" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="D9" s="35">
+      <c r="D9" s="36">
         <v>0.0</v>
       </c>
       <c r="E9" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="40" t="s">
+      <c r="F9" s="41" t="s">
         <v>156</v>
       </c>
     </row>
@@ -4802,7 +4805,7 @@
       <c r="C10" s="27" t="s">
         <v>158</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="37">
         <f>H7+D8+D9</f>
         <v>0.1244444444</v>
       </c>
@@ -4817,7 +4820,7 @@
       <c r="C11" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="D11" s="35">
+      <c r="D11" s="36">
         <v>1440.0</v>
       </c>
       <c r="E11" s="27" t="s">
@@ -4831,14 +4834,14 @@
       <c r="C12" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="D12" s="35">
+      <c r="D12" s="36">
         <f>1440/140000*3600</f>
         <v>37.02857143</v>
       </c>
       <c r="E12" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="40" t="s">
+      <c r="H12" s="41" t="s">
         <v>163</v>
       </c>
       <c r="I12" s="27">
@@ -4853,7 +4856,7 @@
       <c r="C13" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="D13" s="36">
+      <c r="D13" s="37">
         <f>(D12+D11*D10)/60</f>
         <v>3.603809524</v>
       </c>
@@ -4882,34 +4885,34 @@
       <c r="C14" s="27" t="s">
         <v>170</v>
       </c>
-      <c r="D14" s="35">
+      <c r="D14" s="36">
         <f>0.01*1440</f>
         <v>14.4</v>
       </c>
       <c r="E14" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="40" t="s">
+      <c r="F14" s="41" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="42" t="s">
         <v>172</v>
       </c>
-      <c r="C15" s="41" t="s">
+      <c r="C15" s="42" t="s">
         <v>173</v>
       </c>
-      <c r="D15" s="42">
+      <c r="D15" s="43">
         <f>(D14+D13*60)/60</f>
         <v>3.843809524</v>
       </c>
-      <c r="E15" s="41" t="s">
+      <c r="E15" s="42" t="s">
         <v>166</v>
       </c>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="43"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
     </row>
     <row r="16">
       <c r="B16" s="27" t="s">
@@ -4918,7 +4921,7 @@
       <c r="C16" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="D16" s="36">
+      <c r="D16" s="37">
         <f>D13*60/D11</f>
         <v>0.1501587302</v>
       </c>
@@ -4928,22 +4931,22 @@
       <c r="F16" s="27"/>
     </row>
     <row r="17">
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="42" t="s">
         <v>176</v>
       </c>
-      <c r="C17" s="41" t="s">
+      <c r="C17" s="42" t="s">
         <v>177</v>
       </c>
-      <c r="D17" s="42">
+      <c r="D17" s="43">
         <f>3600/D16</f>
         <v>23974.63002</v>
       </c>
-      <c r="E17" s="41" t="s">
+      <c r="E17" s="42" t="s">
         <v>178</v>
       </c>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
     </row>
     <row r="18">
       <c r="B18" s="27" t="s">
@@ -4952,13 +4955,13 @@
       <c r="C18" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="D18" s="35">
+      <c r="D18" s="36">
         <v>2.0</v>
       </c>
       <c r="E18" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="F18" s="44" t="s">
+      <c r="F18" s="45" t="s">
         <v>182</v>
       </c>
     </row>
@@ -4969,7 +4972,7 @@
       <c r="C19" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="D19" s="36">
+      <c r="D19" s="37">
         <f>7*3</f>
         <v>21</v>
       </c>
@@ -4984,7 +4987,7 @@
       <c r="C20" s="27" t="s">
         <v>187</v>
       </c>
-      <c r="D20" s="35">
+      <c r="D20" s="36">
         <v>7.0</v>
       </c>
       <c r="E20" s="27" t="s">
@@ -4992,22 +4995,22 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="41" t="s">
+      <c r="B21" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="D21" s="45">
+      <c r="D21" s="46">
         <f>D18*D19*D20*D17</f>
         <v>7048541.226</v>
       </c>
-      <c r="E21" s="41" t="s">
+      <c r="E21" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="43"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22">
       <c r="B22" s="27" t="s">
@@ -5068,7 +5071,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="47" t="s">
         <v>202</v>
       </c>
       <c r="C26" s="27" t="s">
@@ -5079,7 +5082,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="46" t="s">
+      <c r="B27" s="47" t="s">
         <v>204</v>
       </c>
       <c r="C27" s="27" t="s">
@@ -5090,7 +5093,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="46" t="s">
+      <c r="B28" s="47" t="s">
         <v>206</v>
       </c>
       <c r="C28" s="27" t="s">
@@ -5101,7 +5104,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="46" t="s">
+      <c r="B29" s="47" t="s">
         <v>208</v>
       </c>
       <c r="C29" s="27" t="s">
@@ -5112,7 +5115,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="46" t="s">
+      <c r="B30" s="47" t="s">
         <v>210</v>
       </c>
       <c r="C30" s="27" t="s">
@@ -5123,7 +5126,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="46" t="s">
+      <c r="B31" s="47" t="s">
         <v>212</v>
       </c>
       <c r="C31" s="27" t="s">
@@ -5134,7 +5137,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="46" t="s">
+      <c r="B32" s="47" t="s">
         <v>214</v>
       </c>
       <c r="C32" s="27" t="s">
@@ -5145,7 +5148,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="46" t="s">
+      <c r="B33" s="47" t="s">
         <v>216</v>
       </c>
       <c r="C33" s="27" t="s">
@@ -5156,7 +5159,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="46" t="s">
+      <c r="B34" s="47" t="s">
         <v>218</v>
       </c>
       <c r="C34" s="27" t="s">
@@ -5167,7 +5170,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="46" t="s">
+      <c r="B35" s="47" t="s">
         <v>220</v>
       </c>
       <c r="C35" s="27" t="s">
@@ -5178,7 +5181,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="46" t="s">
+      <c r="B36" s="47" t="s">
         <v>222</v>
       </c>
       <c r="C36" s="27" t="s">
@@ -5189,7 +5192,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="46" t="s">
+      <c r="B37" s="47" t="s">
         <v>224</v>
       </c>
       <c r="C37" s="27" t="s">
@@ -5212,7 +5215,7 @@
       <c r="E38" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="F38" s="40" t="s">
+      <c r="F38" s="41" t="s">
         <v>228</v>
       </c>
     </row>
@@ -5229,27 +5232,27 @@
       <c r="E39" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="F39" s="40" t="s">
+      <c r="F39" s="41" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="41" t="s">
+      <c r="B40" s="42" t="s">
         <v>232</v>
       </c>
-      <c r="C40" s="41" t="s">
+      <c r="C40" s="42" t="s">
         <v>233</v>
       </c>
-      <c r="D40" s="43">
+      <c r="D40" s="44">
         <f>SUM(D24:D39)</f>
         <v>360</v>
       </c>
-      <c r="E40" s="41" t="s">
+      <c r="E40" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="F40" s="43"/>
-      <c r="G40" s="43"/>
-      <c r="H40" s="43"/>
+      <c r="F40" s="44"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="44"/>
     </row>
     <row r="41">
       <c r="B41" s="27" t="s">
@@ -5423,7 +5426,7 @@
       <c r="E50" s="27" t="s">
         <v>256</v>
       </c>
-      <c r="F50" s="40" t="s">
+      <c r="F50" s="41" t="s">
         <v>257</v>
       </c>
     </row>
@@ -5434,14 +5437,14 @@
       <c r="C51" s="27" t="s">
         <v>259</v>
       </c>
-      <c r="D51" s="35">
+      <c r="D51" s="36">
         <f>D45/D50</f>
         <v>0.147275405</v>
       </c>
       <c r="E51" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="F51" s="40" t="s">
+      <c r="F51" s="41" t="s">
         <v>260</v>
       </c>
     </row>
@@ -5452,7 +5455,7 @@
       <c r="C52" s="27" t="s">
         <v>262</v>
       </c>
-      <c r="D52" s="36">
+      <c r="D52" s="37">
         <f>D51*D50/D45</f>
         <v>1</v>
       </c>
@@ -5467,7 +5470,7 @@
       <c r="C53" s="27" t="s">
         <v>264</v>
       </c>
-      <c r="D53" s="47">
+      <c r="D53" s="48">
         <f>D6/D51</f>
         <v>1.2222</v>
       </c>
@@ -5482,7 +5485,7 @@
       <c r="C54" s="27" t="s">
         <v>266</v>
       </c>
-      <c r="D54" s="47">
+      <c r="D54" s="48">
         <f>D52*D53</f>
         <v>1.2222</v>
       </c>
@@ -5501,7 +5504,7 @@
         <f>23000*7*0.03</f>
         <v>4830</v>
       </c>
-      <c r="F55" s="40" t="s">
+      <c r="F55" s="41" t="s">
         <v>269</v>
       </c>
     </row>
@@ -5512,7 +5515,7 @@
       <c r="C56" s="27" t="s">
         <v>271</v>
       </c>
-      <c r="D56" s="47">
+      <c r="D56" s="48">
         <f>(D50-D55)/D50</f>
         <v>0.9708991897</v>
       </c>

</xml_diff>